<commit_message>
added fundamental analysis to the end after the sector selection
</commit_message>
<xml_diff>
--- a/Code/stock.xlsx
+++ b/Code/stock.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lvos2\OneDrive\Desktop\Github Code\PMP_Fundamental\Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B1A4DC1-D9DE-4F99-A2F8-C2A599D04C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460D2D9B-946C-4AE5-B5D6-05CBFFE3A2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4965" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$AN$342</definedName>
+  </definedNames>
   <calcPr calcId="191028" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2781,15 +2784,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AN342"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="44.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="31" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="14" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="16" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:40" x14ac:dyDescent="0.25">
@@ -2914,7 +2952,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -3083,7 +3121,7 @@
         <v>13.4716</v>
       </c>
     </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -3296,7 +3334,7 @@
         <v>12.0998</v>
       </c>
     </row>
-    <row r="7" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -3376,7 +3414,7 @@
         <v>0.49469999999999997</v>
       </c>
     </row>
-    <row r="8" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>63</v>
       </c>
@@ -3471,7 +3509,7 @@
         <v>31.168600000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>68</v>
       </c>
@@ -3548,7 +3586,7 @@
         <v>50.828299999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>71</v>
       </c>
@@ -3640,7 +3678,7 @@
         <v>28.607800000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>76</v>
       </c>
@@ -3794,7 +3832,7 @@
         <v>0.77759999999999996</v>
       </c>
     </row>
-    <row r="13" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>80</v>
       </c>
@@ -3892,7 +3930,7 @@
         <v>38.367899999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>82</v>
       </c>
@@ -3981,7 +4019,7 @@
         <v>30.629899999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>86</v>
       </c>
@@ -4209,7 +4247,7 @@
         <v>124.7989</v>
       </c>
     </row>
-    <row r="18" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -4431,7 +4469,7 @@
         <v>-196.6575</v>
       </c>
     </row>
-    <row r="21" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>99</v>
       </c>
@@ -4594,7 +4632,7 @@
         <v>-9.7799999999999994</v>
       </c>
     </row>
-    <row r="23" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>104</v>
       </c>
@@ -4683,7 +4721,7 @@
         <v>33.457799999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>106</v>
       </c>
@@ -4778,7 +4816,7 @@
         <v>71.379499999999993</v>
       </c>
     </row>
-    <row r="25" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>109</v>
       </c>
@@ -4870,7 +4908,7 @@
         <v>35.4908</v>
       </c>
     </row>
-    <row r="26" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>112</v>
       </c>
@@ -4956,7 +4994,7 @@
         <v>0.59740000000000004</v>
       </c>
     </row>
-    <row r="27" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>114</v>
       </c>
@@ -5116,7 +5154,7 @@
         <v>1.0967</v>
       </c>
     </row>
-    <row r="29" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>119</v>
       </c>
@@ -5217,7 +5255,7 @@
         <v>31.6874</v>
       </c>
     </row>
-    <row r="30" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>124</v>
       </c>
@@ -5303,7 +5341,7 @@
         <v>0.72499999999999998</v>
       </c>
     </row>
-    <row r="31" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>126</v>
       </c>
@@ -5386,7 +5424,7 @@
         <v>63.639000000000003</v>
       </c>
     </row>
-    <row r="32" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>129</v>
       </c>
@@ -5475,7 +5513,7 @@
         <v>4.4884000000000004</v>
       </c>
     </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>132</v>
       </c>
@@ -5516,7 +5554,7 @@
         <v>2.1724999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>134</v>
       </c>
@@ -5599,7 +5637,7 @@
         <v>62.188099999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>137</v>
       </c>
@@ -5830,7 +5868,7 @@
         <v>-16.8872</v>
       </c>
     </row>
-    <row r="38" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>143</v>
       </c>
@@ -5892,7 +5930,7 @@
         <v>19.422000000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>145</v>
       </c>
@@ -5966,7 +6004,7 @@
         <v>10.768000000000001</v>
       </c>
     </row>
-    <row r="40" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>147</v>
       </c>
@@ -6058,7 +6096,7 @@
         <v>15.5524</v>
       </c>
     </row>
-    <row r="41" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>149</v>
       </c>
@@ -6156,7 +6194,7 @@
         <v>67.896600000000007</v>
       </c>
     </row>
-    <row r="42" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>151</v>
       </c>
@@ -6233,7 +6271,7 @@
         <v>-51.5077</v>
       </c>
     </row>
-    <row r="43" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>155</v>
       </c>
@@ -6313,7 +6351,7 @@
         <v>0.70840000000000003</v>
       </c>
     </row>
-    <row r="44" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>158</v>
       </c>
@@ -6544,7 +6582,7 @@
         <v>10.5519</v>
       </c>
     </row>
-    <row r="47" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>164</v>
       </c>
@@ -6636,7 +6674,7 @@
         <v>18.687799999999999</v>
       </c>
     </row>
-    <row r="48" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>166</v>
       </c>
@@ -6680,7 +6718,7 @@
         <v>89.2834</v>
       </c>
     </row>
-    <row r="49" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>168</v>
       </c>
@@ -6751,7 +6789,7 @@
         <v>20.048500000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>170</v>
       </c>
@@ -6840,7 +6878,7 @@
         <v>-2.8431000000000002</v>
       </c>
     </row>
-    <row r="51" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>173</v>
       </c>
@@ -6932,7 +6970,7 @@
         <v>2644.4394000000002</v>
       </c>
     </row>
-    <row r="52" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>175</v>
       </c>
@@ -6988,7 +7026,7 @@
         <v>-9252.2145999999993</v>
       </c>
     </row>
-    <row r="53" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>177</v>
       </c>
@@ -7080,7 +7118,7 @@
         <v>15.627599999999999</v>
       </c>
     </row>
-    <row r="54" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>179</v>
       </c>
@@ -7169,7 +7207,7 @@
         <v>25.172799999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>181</v>
       </c>
@@ -7338,7 +7376,7 @@
         <v>-86.948099999999997</v>
       </c>
     </row>
-    <row r="57" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>186</v>
       </c>
@@ -7486,7 +7524,7 @@
         <v>8.0786999999999995</v>
       </c>
     </row>
-    <row r="59" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>190</v>
       </c>
@@ -7649,7 +7687,7 @@
         <v>13.637499999999999</v>
       </c>
     </row>
-    <row r="61" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>195</v>
       </c>
@@ -7711,7 +7749,7 @@
         <v>23.869299999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>198</v>
       </c>
@@ -7895,7 +7933,7 @@
         <v>122.9499</v>
       </c>
     </row>
-    <row r="64" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>202</v>
       </c>
@@ -7954,7 +7992,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="65" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>204</v>
       </c>
@@ -8031,7 +8069,7 @@
         <v>0.39410000000000001</v>
       </c>
     </row>
-    <row r="66" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>206</v>
       </c>
@@ -8120,7 +8158,7 @@
         <v>44.183</v>
       </c>
     </row>
-    <row r="67" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>208</v>
       </c>
@@ -8191,7 +8229,7 @@
         <v>0.26390000000000002</v>
       </c>
     </row>
-    <row r="68" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>210</v>
       </c>
@@ -8283,7 +8321,7 @@
         <v>56.2074</v>
       </c>
     </row>
-    <row r="69" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>212</v>
       </c>
@@ -8375,7 +8413,7 @@
         <v>40.062800000000003</v>
       </c>
     </row>
-    <row r="70" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>214</v>
       </c>
@@ -8532,7 +8570,7 @@
         <v>-1.8035000000000001</v>
       </c>
     </row>
-    <row r="72" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>219</v>
       </c>
@@ -8624,7 +8662,7 @@
         <v>10.805</v>
       </c>
     </row>
-    <row r="73" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>221</v>
       </c>
@@ -8716,7 +8754,7 @@
         <v>22.948699999999999</v>
       </c>
     </row>
-    <row r="74" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>223</v>
       </c>
@@ -8796,7 +8834,7 @@
         <v>0.47370000000000001</v>
       </c>
     </row>
-    <row r="75" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>225</v>
       </c>
@@ -8873,7 +8911,7 @@
         <v>2.0495999999999999</v>
       </c>
     </row>
-    <row r="76" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>227</v>
       </c>
@@ -8953,7 +8991,7 @@
         <v>0.29980000000000001</v>
       </c>
     </row>
-    <row r="77" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>229</v>
       </c>
@@ -9054,7 +9092,7 @@
         <v>83.832099999999997</v>
       </c>
     </row>
-    <row r="78" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>231</v>
       </c>
@@ -9146,7 +9184,7 @@
         <v>6.8426</v>
       </c>
     </row>
-    <row r="79" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>233</v>
       </c>
@@ -9220,7 +9258,7 @@
         <v>10.528</v>
       </c>
     </row>
-    <row r="80" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>235</v>
       </c>
@@ -9318,7 +9356,7 @@
         <v>17.690899999999999</v>
       </c>
     </row>
-    <row r="81" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>237</v>
       </c>
@@ -9389,7 +9427,7 @@
         <v>28.1143</v>
       </c>
     </row>
-    <row r="82" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>239</v>
       </c>
@@ -9481,7 +9519,7 @@
         <v>48.8095</v>
       </c>
     </row>
-    <row r="83" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>241</v>
       </c>
@@ -9567,7 +9605,7 @@
         <v>35.6633</v>
       </c>
     </row>
-    <row r="84" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>243</v>
       </c>
@@ -9650,7 +9688,7 @@
         <v>35.563499999999998</v>
       </c>
     </row>
-    <row r="85" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>245</v>
       </c>
@@ -9742,7 +9780,7 @@
         <v>55.2483</v>
       </c>
     </row>
-    <row r="86" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>247</v>
       </c>
@@ -9837,7 +9875,7 @@
         <v>21.811699999999998</v>
       </c>
     </row>
-    <row r="87" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>249</v>
       </c>
@@ -10000,7 +10038,7 @@
         <v>-12.3591</v>
       </c>
     </row>
-    <row r="89" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>254</v>
       </c>
@@ -10074,7 +10112,7 @@
         <v>0.31240000000000001</v>
       </c>
     </row>
-    <row r="90" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>256</v>
       </c>
@@ -10376,7 +10414,7 @@
         <v>23.380600000000001</v>
       </c>
     </row>
-    <row r="94" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>264</v>
       </c>
@@ -10408,7 +10446,7 @@
         <v>3.3871000000000002</v>
       </c>
     </row>
-    <row r="95" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>268</v>
       </c>
@@ -10482,7 +10520,7 @@
         <v>0.58630000000000004</v>
       </c>
     </row>
-    <row r="96" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>271</v>
       </c>
@@ -10550,7 +10588,7 @@
         <v>0.55320000000000003</v>
       </c>
     </row>
-    <row r="97" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>273</v>
       </c>
@@ -10689,7 +10727,7 @@
         <v>20.207599999999999</v>
       </c>
     </row>
-    <row r="99" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>278</v>
       </c>
@@ -10769,7 +10807,7 @@
         <v>-74.323400000000007</v>
       </c>
     </row>
-    <row r="100" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>280</v>
       </c>
@@ -10861,7 +10899,7 @@
         <v>44.625900000000001</v>
       </c>
     </row>
-    <row r="101" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>282</v>
       </c>
@@ -10950,7 +10988,7 @@
         <v>47.253599999999999</v>
       </c>
     </row>
-    <row r="102" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>284</v>
       </c>
@@ -11098,7 +11136,7 @@
         <v>-1.7873000000000001</v>
       </c>
     </row>
-    <row r="104" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>288</v>
       </c>
@@ -11178,7 +11216,7 @@
         <v>66.934299999999993</v>
       </c>
     </row>
-    <row r="105" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>290</v>
       </c>
@@ -11264,7 +11302,7 @@
         <v>53.078499999999998</v>
       </c>
     </row>
-    <row r="106" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>292</v>
       </c>
@@ -11347,7 +11385,7 @@
         <v>6.5593000000000004</v>
       </c>
     </row>
-    <row r="107" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>294</v>
       </c>
@@ -11436,7 +11474,7 @@
         <v>73.143500000000003</v>
       </c>
     </row>
-    <row r="108" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>296</v>
       </c>
@@ -11513,7 +11551,7 @@
         <v>-27.1569</v>
       </c>
     </row>
-    <row r="109" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>298</v>
       </c>
@@ -11593,7 +11631,7 @@
         <v>0.39600000000000002</v>
       </c>
     </row>
-    <row r="110" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>300</v>
       </c>
@@ -11685,7 +11723,7 @@
         <v>12.865600000000001</v>
       </c>
     </row>
-    <row r="111" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>302</v>
       </c>
@@ -11818,7 +11856,7 @@
         <v>-8.9848999999999997</v>
       </c>
     </row>
-    <row r="113" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>307</v>
       </c>
@@ -11886,7 +11924,7 @@
         <v>12.0106</v>
       </c>
     </row>
-    <row r="114" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>309</v>
       </c>
@@ -12102,7 +12140,7 @@
         <v>6.9246999999999996</v>
       </c>
     </row>
-    <row r="117" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>315</v>
       </c>
@@ -12197,7 +12235,7 @@
         <v>25.256900000000002</v>
       </c>
     </row>
-    <row r="118" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>317</v>
       </c>
@@ -12292,7 +12330,7 @@
         <v>14.623900000000001</v>
       </c>
     </row>
-    <row r="119" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>319</v>
       </c>
@@ -12446,7 +12484,7 @@
         <v>-3.5434000000000001</v>
       </c>
     </row>
-    <row r="121" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>324</v>
       </c>
@@ -12511,7 +12549,7 @@
         <v>8.1806999999999999</v>
       </c>
     </row>
-    <row r="122" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>326</v>
       </c>
@@ -12641,7 +12679,7 @@
         <v>15.1867</v>
       </c>
     </row>
-    <row r="124" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>330</v>
       </c>
@@ -12783,7 +12821,7 @@
         <v>12.4986</v>
       </c>
     </row>
-    <row r="126" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>334</v>
       </c>
@@ -12872,7 +12910,7 @@
         <v>267.91039999999998</v>
       </c>
     </row>
-    <row r="127" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>336</v>
       </c>
@@ -12940,7 +12978,7 @@
         <v>7.3800000000000004E-2</v>
       </c>
     </row>
-    <row r="128" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>338</v>
       </c>
@@ -13029,7 +13067,7 @@
         <v>1.7491000000000001</v>
       </c>
     </row>
-    <row r="129" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>340</v>
       </c>
@@ -13094,7 +13132,7 @@
         <v>43.897599999999997</v>
       </c>
     </row>
-    <row r="130" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>342</v>
       </c>
@@ -13183,7 +13221,7 @@
         <v>62.435499999999998</v>
       </c>
     </row>
-    <row r="131" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>344</v>
       </c>
@@ -13275,7 +13313,7 @@
         <v>28.903700000000001</v>
       </c>
     </row>
-    <row r="132" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>346</v>
       </c>
@@ -13420,7 +13458,7 @@
         <v>13.209099999999999</v>
       </c>
     </row>
-    <row r="134" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>350</v>
       </c>
@@ -13512,7 +13550,7 @@
         <v>6.0648</v>
       </c>
     </row>
-    <row r="135" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>352</v>
       </c>
@@ -13595,7 +13633,7 @@
         <v>-11.208600000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>354</v>
       </c>
@@ -13681,7 +13719,7 @@
         <v>44.263100000000001</v>
       </c>
     </row>
-    <row r="137" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>356</v>
       </c>
@@ -13776,7 +13814,7 @@
         <v>0.1414</v>
       </c>
     </row>
-    <row r="138" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>358</v>
       </c>
@@ -13865,7 +13903,7 @@
         <v>7.0983999999999998</v>
       </c>
     </row>
-    <row r="139" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>360</v>
       </c>
@@ -14019,7 +14057,7 @@
         <v>0.87370000000000003</v>
       </c>
     </row>
-    <row r="141" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>366</v>
       </c>
@@ -14102,7 +14140,7 @@
         <v>52.283000000000001</v>
       </c>
     </row>
-    <row r="142" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>368</v>
       </c>
@@ -14223,7 +14261,7 @@
         <v>13.6991</v>
       </c>
     </row>
-    <row r="144" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>372</v>
       </c>
@@ -14294,7 +14332,7 @@
         <v>4.8602999999999996</v>
       </c>
     </row>
-    <row r="145" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>374</v>
       </c>
@@ -14374,7 +14412,7 @@
         <v>0.65620000000000001</v>
       </c>
     </row>
-    <row r="146" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>376</v>
       </c>
@@ -14454,7 +14492,7 @@
         <v>30.5745</v>
       </c>
     </row>
-    <row r="147" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>378</v>
       </c>
@@ -14534,7 +14572,7 @@
         <v>0.3987</v>
       </c>
     </row>
-    <row r="148" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>380</v>
       </c>
@@ -14575,7 +14613,7 @@
         <v>1.0528999999999999</v>
       </c>
     </row>
-    <row r="149" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>382</v>
       </c>
@@ -14670,7 +14708,7 @@
         <v>47.802599999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>384</v>
       </c>
@@ -14833,7 +14871,7 @@
         <v>7.8045</v>
       </c>
     </row>
-    <row r="152" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>388</v>
       </c>
@@ -14919,7 +14957,7 @@
         <v>45.828400000000002</v>
       </c>
     </row>
-    <row r="153" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>390</v>
       </c>
@@ -15085,7 +15123,7 @@
         <v>-0.38879999999999998</v>
       </c>
     </row>
-    <row r="155" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>394</v>
       </c>
@@ -15168,7 +15206,7 @@
         <v>3.8959000000000001</v>
       </c>
     </row>
-    <row r="156" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>396</v>
       </c>
@@ -15233,7 +15271,7 @@
         <v>24.6769</v>
       </c>
     </row>
-    <row r="157" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>398</v>
       </c>
@@ -15328,7 +15366,7 @@
         <v>24.799299999999999</v>
       </c>
     </row>
-    <row r="158" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>400</v>
       </c>
@@ -15402,7 +15440,7 @@
         <v>59.229199999999999</v>
       </c>
     </row>
-    <row r="159" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>402</v>
       </c>
@@ -15482,7 +15520,7 @@
         <v>-71.428600000000003</v>
       </c>
     </row>
-    <row r="160" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>404</v>
       </c>
@@ -15565,7 +15603,7 @@
         <v>35.375300000000003</v>
       </c>
     </row>
-    <row r="161" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>406</v>
       </c>
@@ -15645,7 +15683,7 @@
         <v>42.623100000000001</v>
       </c>
     </row>
-    <row r="162" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>408</v>
       </c>
@@ -15725,7 +15763,7 @@
         <v>28.335100000000001</v>
       </c>
     </row>
-    <row r="163" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>410</v>
       </c>
@@ -15811,7 +15849,7 @@
         <v>12.622400000000001</v>
       </c>
     </row>
-    <row r="164" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>412</v>
       </c>
@@ -15909,7 +15947,7 @@
         <v>14.473000000000001</v>
       </c>
     </row>
-    <row r="165" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>414</v>
       </c>
@@ -15986,7 +16024,7 @@
         <v>0.63109999999999999</v>
       </c>
     </row>
-    <row r="166" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>416</v>
       </c>
@@ -16063,7 +16101,7 @@
         <v>1.0951</v>
       </c>
     </row>
-    <row r="167" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>418</v>
       </c>
@@ -16226,7 +16264,7 @@
         <v>28.041</v>
       </c>
     </row>
-    <row r="169" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>422</v>
       </c>
@@ -16318,7 +16356,7 @@
         <v>19.7379</v>
       </c>
     </row>
-    <row r="170" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>424</v>
       </c>
@@ -16407,7 +16445,7 @@
         <v>10.679500000000001</v>
       </c>
     </row>
-    <row r="171" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>426</v>
       </c>
@@ -16623,7 +16661,7 @@
         <v>20.0151</v>
       </c>
     </row>
-    <row r="174" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>432</v>
       </c>
@@ -16694,7 +16732,7 @@
         <v>71.376499999999993</v>
       </c>
     </row>
-    <row r="175" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>434</v>
       </c>
@@ -16780,7 +16818,7 @@
         <v>-6.5343</v>
       </c>
     </row>
-    <row r="176" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>436</v>
       </c>
@@ -16872,7 +16910,7 @@
         <v>13.1409</v>
       </c>
     </row>
-    <row r="177" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>438</v>
       </c>
@@ -17038,7 +17076,7 @@
         <v>-14.0152</v>
       </c>
     </row>
-    <row r="179" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>442</v>
       </c>
@@ -17139,7 +17177,7 @@
         <v>82.6965</v>
       </c>
     </row>
-    <row r="180" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>444</v>
       </c>
@@ -17231,7 +17269,7 @@
         <v>2.5215999999999998</v>
       </c>
     </row>
-    <row r="181" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>446</v>
       </c>
@@ -17364,7 +17402,7 @@
         <v>-6.9084000000000003</v>
       </c>
     </row>
-    <row r="183" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>451</v>
       </c>
@@ -17456,7 +17494,7 @@
         <v>52.024500000000003</v>
       </c>
     </row>
-    <row r="184" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>453</v>
       </c>
@@ -17530,7 +17568,7 @@
         <v>0.4204</v>
       </c>
     </row>
-    <row r="185" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>455</v>
       </c>
@@ -17592,7 +17630,7 @@
         <v>-4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="186" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>457</v>
       </c>
@@ -17832,7 +17870,7 @@
         <v>-2.1987999999999999</v>
       </c>
     </row>
-    <row r="189" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>463</v>
       </c>
@@ -17912,7 +17950,7 @@
         <v>0.45090000000000002</v>
       </c>
     </row>
-    <row r="190" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>465</v>
       </c>
@@ -17986,7 +18024,7 @@
         <v>-5.7272999999999996</v>
       </c>
     </row>
-    <row r="191" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>467</v>
       </c>
@@ -18069,7 +18107,7 @@
         <v>21.107099999999999</v>
       </c>
     </row>
-    <row r="192" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>469</v>
       </c>
@@ -18155,7 +18193,7 @@
         <v>47.133800000000001</v>
       </c>
     </row>
-    <row r="193" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>471</v>
       </c>
@@ -18303,7 +18341,7 @@
         <v>10.114000000000001</v>
       </c>
     </row>
-    <row r="195" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>475</v>
       </c>
@@ -18389,7 +18427,7 @@
         <v>20.7822</v>
       </c>
     </row>
-    <row r="196" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>477</v>
       </c>
@@ -18555,7 +18593,7 @@
         <v>27.585699999999999</v>
       </c>
     </row>
-    <row r="198" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>482</v>
       </c>
@@ -18638,7 +18676,7 @@
         <v>2.3500999999999999</v>
       </c>
     </row>
-    <row r="199" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>484</v>
       </c>
@@ -18682,7 +18720,7 @@
         <v>56.497599999999998</v>
       </c>
     </row>
-    <row r="200" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>486</v>
       </c>
@@ -18780,7 +18818,7 @@
         <v>16.490100000000002</v>
       </c>
     </row>
-    <row r="201" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>488</v>
       </c>
@@ -18860,7 +18898,7 @@
         <v>0.47539999999999999</v>
       </c>
     </row>
-    <row r="202" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>490</v>
       </c>
@@ -18940,7 +18978,7 @@
         <v>0.38729999999999998</v>
       </c>
     </row>
-    <row r="203" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>492</v>
       </c>
@@ -19020,7 +19058,7 @@
         <v>13.8347</v>
       </c>
     </row>
-    <row r="204" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>494</v>
       </c>
@@ -19103,7 +19141,7 @@
         <v>26.833500000000001</v>
       </c>
     </row>
-    <row r="205" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>496</v>
       </c>
@@ -19254,7 +19292,7 @@
         <v>-11.943899999999999</v>
       </c>
     </row>
-    <row r="207" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>500</v>
       </c>
@@ -19565,7 +19603,7 @@
         <v>-130.06299999999999</v>
       </c>
     </row>
-    <row r="211" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>508</v>
       </c>
@@ -19713,7 +19751,7 @@
         <v>18.072399999999998</v>
       </c>
     </row>
-    <row r="213" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>513</v>
       </c>
@@ -19861,7 +19899,7 @@
         <v>8.0633999999999997</v>
       </c>
     </row>
-    <row r="215" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>517</v>
       </c>
@@ -19947,7 +19985,7 @@
         <v>45.865400000000001</v>
       </c>
     </row>
-    <row r="216" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>519</v>
       </c>
@@ -20027,7 +20065,7 @@
         <v>-116.36069999999999</v>
       </c>
     </row>
-    <row r="217" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>522</v>
       </c>
@@ -20101,7 +20139,7 @@
         <v>0.253</v>
       </c>
     </row>
-    <row r="218" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>524</v>
       </c>
@@ -20255,7 +20293,7 @@
         <v>-1.7322</v>
       </c>
     </row>
-    <row r="220" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>528</v>
       </c>
@@ -20329,7 +20367,7 @@
         <v>-580.21720000000005</v>
       </c>
     </row>
-    <row r="221" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>530</v>
       </c>
@@ -20409,7 +20447,7 @@
         <v>0.39539999999999997</v>
       </c>
     </row>
-    <row r="222" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>532</v>
       </c>
@@ -20489,7 +20527,7 @@
         <v>16.470400000000001</v>
       </c>
     </row>
-    <row r="223" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>534</v>
       </c>
@@ -20560,7 +20598,7 @@
         <v>20.552900000000001</v>
       </c>
     </row>
-    <row r="224" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>536</v>
       </c>
@@ -20640,7 +20678,7 @@
         <v>0.37290000000000001</v>
       </c>
     </row>
-    <row r="225" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>538</v>
       </c>
@@ -20735,7 +20773,7 @@
         <v>8.1723999999999997</v>
       </c>
     </row>
-    <row r="226" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>540</v>
       </c>
@@ -20809,7 +20847,7 @@
         <v>21.361799999999999</v>
       </c>
     </row>
-    <row r="227" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>542</v>
       </c>
@@ -21064,7 +21102,7 @@
         <v>-5.3529</v>
       </c>
     </row>
-    <row r="230" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>548</v>
       </c>
@@ -21162,7 +21200,7 @@
         <v>21.037199999999999</v>
       </c>
     </row>
-    <row r="231" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>550</v>
       </c>
@@ -21251,7 +21289,7 @@
         <v>39.136299999999999</v>
       </c>
     </row>
-    <row r="232" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>552</v>
       </c>
@@ -21429,7 +21467,7 @@
         <v>52.792499999999997</v>
       </c>
     </row>
-    <row r="234" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>556</v>
       </c>
@@ -21592,7 +21630,7 @@
         <v>4.3837999999999999</v>
       </c>
     </row>
-    <row r="236" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>562</v>
       </c>
@@ -21681,7 +21719,7 @@
         <v>59.298499999999997</v>
       </c>
     </row>
-    <row r="237" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>564</v>
       </c>
@@ -21862,7 +21900,7 @@
         <v>12.001300000000001</v>
       </c>
     </row>
-    <row r="239" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>568</v>
       </c>
@@ -21936,7 +21974,7 @@
         <v>13.2493</v>
       </c>
     </row>
-    <row r="240" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>570</v>
       </c>
@@ -22019,7 +22057,7 @@
         <v>0.4909</v>
       </c>
     </row>
-    <row r="241" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>572</v>
       </c>
@@ -22161,7 +22199,7 @@
         <v>-23.503599999999999</v>
       </c>
     </row>
-    <row r="243" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>576</v>
       </c>
@@ -22250,7 +22288,7 @@
         <v>60.418300000000002</v>
       </c>
     </row>
-    <row r="244" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>578</v>
       </c>
@@ -22413,7 +22451,7 @@
         <v>9.0641999999999996</v>
       </c>
     </row>
-    <row r="246" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>582</v>
       </c>
@@ -22493,7 +22531,7 @@
         <v>22.781199999999998</v>
       </c>
     </row>
-    <row r="247" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>584</v>
       </c>
@@ -22582,7 +22620,7 @@
         <v>-26.128799999999998</v>
       </c>
     </row>
-    <row r="248" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>586</v>
       </c>
@@ -22866,7 +22904,7 @@
         <v>1.9147000000000001</v>
       </c>
     </row>
-    <row r="252" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>594</v>
       </c>
@@ -22913,7 +22951,7 @@
         <v>0.93010000000000004</v>
       </c>
     </row>
-    <row r="253" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>596</v>
       </c>
@@ -22999,7 +23037,7 @@
         <v>9.1336999999999993</v>
       </c>
     </row>
-    <row r="254" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>601</v>
       </c>
@@ -23091,7 +23129,7 @@
         <v>33.633499999999998</v>
       </c>
     </row>
-    <row r="255" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>606</v>
       </c>
@@ -23186,7 +23224,7 @@
         <v>15.9788</v>
       </c>
     </row>
-    <row r="256" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>608</v>
       </c>
@@ -23254,7 +23292,7 @@
         <v>12.2996</v>
       </c>
     </row>
-    <row r="257" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>611</v>
       </c>
@@ -23352,7 +23390,7 @@
         <v>5.8808999999999996</v>
       </c>
     </row>
-    <row r="258" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>613</v>
       </c>
@@ -23426,7 +23464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="259" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>615</v>
       </c>
@@ -23512,7 +23550,7 @@
         <v>-5.0091000000000001</v>
       </c>
     </row>
-    <row r="260" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>619</v>
       </c>
@@ -23586,7 +23624,7 @@
         <v>10.2273</v>
       </c>
     </row>
-    <row r="261" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>621</v>
       </c>
@@ -23669,7 +23707,7 @@
         <v>8.3693000000000008</v>
       </c>
     </row>
-    <row r="262" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>623</v>
       </c>
@@ -23755,7 +23793,7 @@
         <v>28.0625</v>
       </c>
     </row>
-    <row r="263" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>625</v>
       </c>
@@ -23850,7 +23888,7 @@
         <v>28.4831</v>
       </c>
     </row>
-    <row r="264" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>629</v>
       </c>
@@ -23942,7 +23980,7 @@
         <v>8.7314000000000007</v>
       </c>
     </row>
-    <row r="265" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>631</v>
       </c>
@@ -23986,7 +24024,7 @@
         <v>-35.846699999999998</v>
       </c>
     </row>
-    <row r="266" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>636</v>
       </c>
@@ -24081,7 +24119,7 @@
         <v>20.5122</v>
       </c>
     </row>
-    <row r="267" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>639</v>
       </c>
@@ -24170,7 +24208,7 @@
         <v>13.000299999999999</v>
       </c>
     </row>
-    <row r="268" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>641</v>
       </c>
@@ -24253,7 +24291,7 @@
         <v>11.609</v>
       </c>
     </row>
-    <row r="269" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>643</v>
       </c>
@@ -24339,7 +24377,7 @@
         <v>-41.673999999999999</v>
       </c>
     </row>
-    <row r="270" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>648</v>
       </c>
@@ -24434,7 +24472,7 @@
         <v>20.288699999999999</v>
       </c>
     </row>
-    <row r="271" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>650</v>
       </c>
@@ -24517,7 +24555,7 @@
         <v>30.624400000000001</v>
       </c>
     </row>
-    <row r="272" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>653</v>
       </c>
@@ -24612,7 +24650,7 @@
         <v>2.7892999999999999</v>
       </c>
     </row>
-    <row r="273" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>655</v>
       </c>
@@ -24698,7 +24736,7 @@
         <v>5.3612000000000002</v>
       </c>
     </row>
-    <row r="274" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>657</v>
       </c>
@@ -24781,7 +24819,7 @@
         <v>51.901600000000002</v>
       </c>
     </row>
-    <row r="275" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>659</v>
       </c>
@@ -24870,7 +24908,7 @@
         <v>3.6619999999999999</v>
       </c>
     </row>
-    <row r="276" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>661</v>
       </c>
@@ -24968,7 +25006,7 @@
         <v>26.045300000000001</v>
       </c>
     </row>
-    <row r="277" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>663</v>
       </c>
@@ -25054,7 +25092,7 @@
         <v>2.6303999999999998</v>
       </c>
     </row>
-    <row r="278" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>665</v>
       </c>
@@ -25152,7 +25190,7 @@
         <v>24.5732</v>
       </c>
     </row>
-    <row r="279" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>667</v>
       </c>
@@ -25244,7 +25282,7 @@
         <v>23.45</v>
       </c>
     </row>
-    <row r="280" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>669</v>
       </c>
@@ -25339,7 +25377,7 @@
         <v>22.946100000000001</v>
       </c>
     </row>
-    <row r="281" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>674</v>
       </c>
@@ -25431,7 +25469,7 @@
         <v>3.6154999999999999</v>
       </c>
     </row>
-    <row r="282" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>676</v>
       </c>
@@ -25523,7 +25561,7 @@
         <v>11.260899999999999</v>
       </c>
     </row>
-    <row r="283" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>678</v>
       </c>
@@ -25603,7 +25641,7 @@
         <v>-5194.6773999999996</v>
       </c>
     </row>
-    <row r="284" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>680</v>
       </c>
@@ -25659,7 +25697,7 @@
         <v>15.396599999999999</v>
       </c>
     </row>
-    <row r="285" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>682</v>
       </c>
@@ -25745,7 +25783,7 @@
         <v>-7.1586999999999996</v>
       </c>
     </row>
-    <row r="286" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>684</v>
       </c>
@@ -25828,7 +25866,7 @@
         <v>3.5366</v>
       </c>
     </row>
-    <row r="287" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>686</v>
       </c>
@@ -25917,7 +25955,7 @@
         <v>8.9467999999999996</v>
       </c>
     </row>
-    <row r="288" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>688</v>
       </c>
@@ -26003,7 +26041,7 @@
         <v>-5.9076000000000004</v>
       </c>
     </row>
-    <row r="289" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>690</v>
       </c>
@@ -26092,7 +26130,7 @@
         <v>7.6111000000000004</v>
       </c>
     </row>
-    <row r="290" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>692</v>
       </c>
@@ -26178,7 +26216,7 @@
         <v>32.082299999999996</v>
       </c>
     </row>
-    <row r="291" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>694</v>
       </c>
@@ -26264,7 +26302,7 @@
         <v>-6.7552000000000003</v>
       </c>
     </row>
-    <row r="292" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>696</v>
       </c>
@@ -26338,7 +26376,7 @@
         <v>-20.401</v>
       </c>
     </row>
-    <row r="293" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>698</v>
       </c>
@@ -26439,7 +26477,7 @@
         <v>29.787099999999999</v>
       </c>
     </row>
-    <row r="294" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>700</v>
       </c>
@@ -26525,7 +26563,7 @@
         <v>12.911099999999999</v>
       </c>
     </row>
-    <row r="295" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>702</v>
       </c>
@@ -26605,7 +26643,7 @@
         <v>4.4848999999999997</v>
       </c>
     </row>
-    <row r="296" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>704</v>
       </c>
@@ -26700,7 +26738,7 @@
         <v>18.510200000000001</v>
       </c>
     </row>
-    <row r="297" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>706</v>
       </c>
@@ -26786,7 +26824,7 @@
         <v>16.755600000000001</v>
       </c>
     </row>
-    <row r="298" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>708</v>
       </c>
@@ -26881,7 +26919,7 @@
         <v>9.7619000000000007</v>
       </c>
     </row>
-    <row r="299" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>710</v>
       </c>
@@ -26958,7 +26996,7 @@
         <v>-7.5298999999999996</v>
       </c>
     </row>
-    <row r="300" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>712</v>
       </c>
@@ -27029,7 +27067,7 @@
         <v>-6.2544000000000004</v>
       </c>
     </row>
-    <row r="301" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>714</v>
       </c>
@@ -27121,7 +27159,7 @@
         <v>18.3261</v>
       </c>
     </row>
-    <row r="302" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>716</v>
       </c>
@@ -27210,7 +27248,7 @@
         <v>-8.3389000000000006</v>
       </c>
     </row>
-    <row r="303" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>718</v>
       </c>
@@ -27302,7 +27340,7 @@
         <v>10.982200000000001</v>
       </c>
     </row>
-    <row r="304" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>720</v>
       </c>
@@ -27388,7 +27426,7 @@
         <v>-6.0712999999999999</v>
       </c>
     </row>
-    <row r="305" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>722</v>
       </c>
@@ -27471,7 +27509,7 @@
         <v>-9.6166</v>
       </c>
     </row>
-    <row r="306" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>724</v>
       </c>
@@ -27572,7 +27610,7 @@
         <v>19.518699999999999</v>
       </c>
     </row>
-    <row r="307" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>726</v>
       </c>
@@ -27664,7 +27702,7 @@
         <v>14.156499999999999</v>
       </c>
     </row>
-    <row r="308" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>728</v>
       </c>
@@ -27741,7 +27779,7 @@
         <v>-22.7468</v>
       </c>
     </row>
-    <row r="309" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>730</v>
       </c>
@@ -27782,7 +27820,7 @@
         <v>154.22219999999999</v>
       </c>
     </row>
-    <row r="310" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>733</v>
       </c>
@@ -27880,7 +27918,7 @@
         <v>30.2087</v>
       </c>
     </row>
-    <row r="311" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>735</v>
       </c>
@@ -27948,7 +27986,7 @@
         <v>-1.5599999999999999E-2</v>
       </c>
     </row>
-    <row r="312" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>738</v>
       </c>
@@ -28040,7 +28078,7 @@
         <v>21.0153</v>
       </c>
     </row>
-    <row r="313" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>740</v>
       </c>
@@ -28132,7 +28170,7 @@
         <v>30.784099999999999</v>
       </c>
     </row>
-    <row r="314" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>742</v>
       </c>
@@ -28212,7 +28250,7 @@
         <v>29.347200000000001</v>
       </c>
     </row>
-    <row r="315" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>744</v>
       </c>
@@ -28271,7 +28309,7 @@
         <v>3.9883000000000002</v>
       </c>
     </row>
-    <row r="316" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>746</v>
       </c>
@@ -28351,7 +28389,7 @@
         <v>33.337000000000003</v>
       </c>
     </row>
-    <row r="317" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>748</v>
       </c>
@@ -28431,7 +28469,7 @@
         <v>-43.2333</v>
       </c>
     </row>
-    <row r="318" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>750</v>
       </c>
@@ -28523,7 +28561,7 @@
         <v>10.938499999999999</v>
       </c>
     </row>
-    <row r="319" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>752</v>
       </c>
@@ -28609,7 +28647,7 @@
         <v>2.5045999999999999</v>
       </c>
     </row>
-    <row r="320" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>754</v>
       </c>
@@ -28704,7 +28742,7 @@
         <v>25.569400000000002</v>
       </c>
     </row>
-    <row r="321" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>756</v>
       </c>
@@ -28799,7 +28837,7 @@
         <v>37.387300000000003</v>
       </c>
     </row>
-    <row r="322" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>758</v>
       </c>
@@ -28870,7 +28908,7 @@
         <v>-182.66749999999999</v>
       </c>
     </row>
-    <row r="323" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>760</v>
       </c>
@@ -28965,7 +29003,7 @@
         <v>6.0045999999999999</v>
       </c>
     </row>
-    <row r="324" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>762</v>
       </c>
@@ -29057,7 +29095,7 @@
         <v>13.2745</v>
       </c>
     </row>
-    <row r="325" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>765</v>
       </c>
@@ -29143,7 +29181,7 @@
         <v>1.016</v>
       </c>
     </row>
-    <row r="326" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>767</v>
       </c>
@@ -29205,7 +29243,7 @@
         <v>10.305999999999999</v>
       </c>
     </row>
-    <row r="327" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>771</v>
       </c>
@@ -29300,7 +29338,7 @@
         <v>27.977799999999998</v>
       </c>
     </row>
-    <row r="328" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>773</v>
       </c>
@@ -29380,7 +29418,7 @@
         <v>21.5167</v>
       </c>
     </row>
-    <row r="329" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>775</v>
       </c>
@@ -29475,7 +29513,7 @@
         <v>18.848700000000001</v>
       </c>
     </row>
-    <row r="330" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>777</v>
       </c>
@@ -29555,7 +29593,7 @@
         <v>-42.090699999999998</v>
       </c>
     </row>
-    <row r="331" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>779</v>
       </c>
@@ -29647,7 +29685,7 @@
         <v>26.508900000000001</v>
       </c>
     </row>
-    <row r="332" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>781</v>
       </c>
@@ -29727,7 +29765,7 @@
         <v>15.028</v>
       </c>
     </row>
-    <row r="333" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>783</v>
       </c>
@@ -29822,7 +29860,7 @@
         <v>13.922700000000001</v>
       </c>
     </row>
-    <row r="334" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>785</v>
       </c>
@@ -29896,7 +29934,7 @@
         <v>-2.6953</v>
       </c>
     </row>
-    <row r="335" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>787</v>
       </c>
@@ -29973,7 +30011,7 @@
         <v>-127.7148</v>
       </c>
     </row>
-    <row r="336" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>789</v>
       </c>
@@ -30062,7 +30100,7 @@
         <v>24.575800000000001</v>
       </c>
     </row>
-    <row r="337" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>791</v>
       </c>
@@ -30133,7 +30171,7 @@
         <v>2.8485999999999998</v>
       </c>
     </row>
-    <row r="338" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>793</v>
       </c>
@@ -30225,7 +30263,7 @@
         <v>37.8185</v>
       </c>
     </row>
-    <row r="339" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>795</v>
       </c>
@@ -30302,7 +30340,7 @@
         <v>35.740400000000001</v>
       </c>
     </row>
-    <row r="340" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>798</v>
       </c>
@@ -30397,7 +30435,7 @@
         <v>7.0857000000000001</v>
       </c>
     </row>
-    <row r="341" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>800</v>
       </c>
@@ -30492,7 +30530,7 @@
         <v>20.505600000000001</v>
       </c>
     </row>
-    <row r="342" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>802</v>
       </c>
@@ -30585,15 +30623,25 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AN342" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Insurance"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -30735,19 +30783,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{692493B9-0457-47C0-897F-1DDBA0309E82}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4DE5A16-F20C-4548-81A2-61017F3EEC82}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -30771,9 +30815,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4DE5A16-F20C-4548-81A2-61017F3EEC82}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{692493B9-0457-47C0-897F-1DDBA0309E82}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>